<commit_message>
Corrects double counting certain capex costs.
</commit_message>
<xml_diff>
--- a/InputData/elec/ASCAPEX/Annual Sustaining CAPEX by Generator Age.xlsx
+++ b/InputData/elec/ASCAPEX/Annual Sustaining CAPEX by Generator Age.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -515,7 +514,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="B10" s="5" t="inlineStr">
         <is>
@@ -544,8 +542,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
@@ -574,6 +570,30 @@
       <c r="B18" s="3" t="inlineStr">
         <is>
           <t>Types without documented age terms (everything except coal/lignite, nuclear, and wind) get a flat base with zero slope/adders - behavior unchanged, and the fallback for regions without vintage data. SMR and hydrogen techs are deliberately flat (no old vintages).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Correction 2026-08-26 (base values only; slopes/adders unchanged):</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>The original bases for nuclear, SMR, and the coal/lignite family were the fleet-weighted ACAPEXpUC constants from the CCaMC workbook. Those constants already embed the fleet's age costs (nuclear: the &gt;30-yr adder, since the whole fleet is &gt;30; coal: ~43-yr capacity-weighted average age x the age slope), so adding the age terms on top double-counted them (~$88k/MW-yr for aged nuclear vs the documented $55.5k).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Bases reset to the EIA age-0 values per this sheet's own documented method: nuclear and SMR = 28 x 0.8287 = 23,203.60 $/MW-yr; hard coal / lignite (+CCS variants) = (16.53 + 5.68 x 0.654 fleet FGD share) x 0.921 = 18645.39 $/MW-yr. FGD share is capacity-weighted from CCaMC 'Annual CAPEX Calcs' (565 coal units, 227 GW). SMR note: its old flat constant simply copied aged-fleet nuclear; a new-build tech is set to the age-0 EIA base for consistency.</t>
         </is>
       </c>
     </row>
@@ -611,7 +631,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>24015.21</v>
+        <v>18645.39</v>
       </c>
     </row>
     <row r="3">
@@ -643,7 +663,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>55528.12</v>
+        <v>23203.6</v>
       </c>
     </row>
     <row r="6">
@@ -743,7 +763,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>24015.21</v>
+        <v>18645.39</v>
       </c>
     </row>
     <row r="15">
@@ -797,7 +817,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>24015.21</v>
+        <v>18645.39</v>
       </c>
     </row>
     <row r="20">
@@ -829,7 +849,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>24015.21</v>
+        <v>18645.39</v>
       </c>
     </row>
     <row r="23">
@@ -839,7 +859,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>55528.12</v>
+        <v>23203.6</v>
       </c>
     </row>
     <row r="24">

</xml_diff>